<commit_message>
improving on NLP. Starting to pack results
</commit_message>
<xml_diff>
--- a/apps_nicolo/MAK_4s_7r_NLP_MAK_REINFORCE/MAK_3s_5r_NLP_MAK_REINFORCE_SIL_COUNCIL.xlsx
+++ b/apps_nicolo/MAK_4s_7r_NLP_MAK_REINFORCE/MAK_3s_5r_NLP_MAK_REINFORCE_SIL_COUNCIL.xlsx
@@ -9,7 +9,7 @@
     <sheet name="Data" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Data'!$A$1:$Z$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Data'!$A$1:$Z$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,6 +30,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color rgb="FF000000"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -60,16 +66,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general"/>
     </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
+      <alignment horizontal="general"/>
     </xf>
     <xf numFmtId="4" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
@@ -77,10 +80,16 @@
     <xf numFmtId="3" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -454,30 +463,30 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z12"/>
+  <dimension ref="A1:Z13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" bestFit="1" customWidth="1" style="7" min="1" max="1"/>
     <col width="14.14785714285714" bestFit="1" customWidth="1" style="7" min="2" max="2"/>
-    <col width="18" bestFit="1" customWidth="1" style="7" min="3" max="3"/>
+    <col width="18" bestFit="1" customWidth="1" style="8" min="3" max="3"/>
     <col width="12" bestFit="1" customWidth="1" style="7" min="4" max="4"/>
     <col width="7" bestFit="1" customWidth="1" style="7" min="5" max="5"/>
     <col width="38" bestFit="1" customWidth="1" style="7" min="6" max="6"/>
-    <col width="15" bestFit="1" customWidth="1" style="8" min="7" max="7"/>
-    <col width="10" bestFit="1" customWidth="1" style="9" min="8" max="8"/>
+    <col width="15" bestFit="1" customWidth="1" style="9" min="7" max="7"/>
+    <col width="10" bestFit="1" customWidth="1" style="10" min="8" max="8"/>
     <col width="17" bestFit="1" customWidth="1" style="7" min="9" max="9"/>
-    <col width="10" bestFit="1" customWidth="1" style="9" min="10" max="10"/>
-    <col width="10" bestFit="1" customWidth="1" style="9" min="11" max="11"/>
-    <col width="17" bestFit="1" customWidth="1" style="9" min="12" max="12"/>
-    <col width="8" bestFit="1" customWidth="1" style="9" min="13" max="13"/>
+    <col width="10" bestFit="1" customWidth="1" style="10" min="10" max="10"/>
+    <col width="10" bestFit="1" customWidth="1" style="10" min="11" max="11"/>
+    <col width="17" bestFit="1" customWidth="1" style="10" min="12" max="12"/>
+    <col width="8" bestFit="1" customWidth="1" style="10" min="13" max="13"/>
     <col width="178" bestFit="1" customWidth="1" style="7" min="14" max="14"/>
     <col width="75" bestFit="1" customWidth="1" style="7" min="15" max="15"/>
-    <col width="17" bestFit="1" customWidth="1" style="9" min="16" max="16"/>
-    <col width="10" bestFit="1" customWidth="1" style="9" min="17" max="17"/>
-    <col width="17" bestFit="1" customWidth="1" style="9" min="18" max="18"/>
-    <col width="14" bestFit="1" customWidth="1" style="9" min="19" max="19"/>
-    <col width="22" bestFit="1" customWidth="1" style="9" min="20" max="20"/>
-    <col width="18" bestFit="1" customWidth="1" style="9" min="21" max="21"/>
+    <col width="17" bestFit="1" customWidth="1" style="10" min="16" max="16"/>
+    <col width="10" bestFit="1" customWidth="1" style="10" min="17" max="17"/>
+    <col width="17" bestFit="1" customWidth="1" style="10" min="18" max="18"/>
+    <col width="14" bestFit="1" customWidth="1" style="10" min="19" max="19"/>
+    <col width="22" bestFit="1" customWidth="1" style="10" min="20" max="20"/>
+    <col width="18" bestFit="1" customWidth="1" style="10" min="21" max="21"/>
     <col width="26" bestFit="1" customWidth="1" style="7" min="22" max="22"/>
     <col width="80" bestFit="1" customWidth="1" style="7" min="23" max="23"/>
     <col width="135" bestFit="1" customWidth="1" style="7" min="24" max="24"/>
@@ -496,7 +505,7 @@
           <t>URL</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
+      <c r="C1" s="8" t="inlineStr">
         <is>
           <t>Epochs Completed</t>
         </is>
@@ -516,12 +525,12 @@
           <t>Comments</t>
         </is>
       </c>
-      <c r="G1" s="8" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Learning Rate</t>
         </is>
       </c>
-      <c r="H1" s="9" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>Epochs #</t>
         </is>
@@ -531,22 +540,22 @@
           <t>(m, n, p, N)</t>
         </is>
       </c>
-      <c r="J1" s="9" t="inlineStr">
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>NN Depth</t>
         </is>
       </c>
-      <c r="K1" s="9" t="inlineStr">
+      <c r="K1" s="4" t="inlineStr">
         <is>
           <t>NN Width</t>
         </is>
       </c>
-      <c r="L1" s="9" t="inlineStr">
+      <c r="L1" s="4" t="inlineStr">
         <is>
           <t>Deep Layer Size</t>
         </is>
       </c>
-      <c r="M1" s="9" t="inlineStr">
+      <c r="M1" s="4" t="inlineStr">
         <is>
           <t>CPUs #</t>
         </is>
@@ -561,32 +570,32 @@
           <t>Risk Scheduler</t>
         </is>
       </c>
-      <c r="P1" s="9" t="inlineStr">
+      <c r="P1" s="4" t="inlineStr">
         <is>
           <t>Render Schedule</t>
         </is>
       </c>
-      <c r="Q1" s="9" t="inlineStr">
+      <c r="Q1" s="4" t="inlineStr">
         <is>
           <t>HoF Size</t>
         </is>
       </c>
-      <c r="R1" s="9" t="inlineStr">
+      <c r="R1" s="4" t="inlineStr">
         <is>
           <t>Simulation Time</t>
         </is>
       </c>
-      <c r="S1" s="9" t="inlineStr">
+      <c r="S1" s="4" t="inlineStr">
         <is>
           <t>Time Steps #</t>
         </is>
       </c>
-      <c r="T1" s="9" t="inlineStr">
+      <c r="T1" s="4" t="inlineStr">
         <is>
           <t>Initial Conditions #</t>
         </is>
       </c>
-      <c r="U1" s="9" t="inlineStr">
+      <c r="U1" s="4" t="inlineStr">
         <is>
           <t>Input Scenarios#</t>
         </is>
@@ -628,14 +637,14 @@
           <t>https://www.comet.com/redsnic/mak-3s-5r-nlp-mak-reinforce-sil-council/f38c5e649f3b4c14b7e761356bf9808a</t>
         </is>
       </c>
-      <c r="C2" s="7" t="n"/>
+      <c r="C2" s="8" t="n"/>
       <c r="D2" s="7" t="n"/>
       <c r="E2" s="7" t="n"/>
       <c r="F2" s="7" t="n"/>
-      <c r="G2" s="4" t="n">
+      <c r="G2" s="5" t="n">
         <v>0.0001</v>
       </c>
-      <c r="H2" s="5" t="n">
+      <c r="H2" s="6" t="n">
         <v>300</v>
       </c>
       <c r="I2" s="7" t="inlineStr">
@@ -643,16 +652,16 @@
           <t>(5, 3, 2, 1280)</t>
         </is>
       </c>
-      <c r="J2" s="5" t="n">
+      <c r="J2" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="K2" s="5" t="n">
+      <c r="K2" s="6" t="n">
         <v>1024</v>
       </c>
-      <c r="L2" s="5" t="n">
+      <c r="L2" s="6" t="n">
         <v>10240</v>
       </c>
-      <c r="M2" s="5" t="n">
+      <c r="M2" s="6" t="n">
         <v>128</v>
       </c>
       <c r="N2" s="7" t="inlineStr">
@@ -665,22 +674,22 @@
           <t>{'risk': 0.9, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
         </is>
       </c>
-      <c r="P2" s="5" t="n">
+      <c r="P2" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="Q2" s="5" t="n">
-        <v>100</v>
-      </c>
-      <c r="R2" s="5" t="n">
-        <v>100</v>
-      </c>
-      <c r="S2" s="5" t="n">
+      <c r="Q2" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="R2" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="S2" s="6" t="n">
         <v>1000</v>
       </c>
-      <c r="T2" s="5" t="n">
+      <c r="T2" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="U2" s="5" t="n">
+      <c r="U2" s="6" t="n">
         <v>9</v>
       </c>
       <c r="V2" s="7" t="inlineStr">
@@ -720,14 +729,14 @@
           <t>https://www.comet.com/redsnic/mak-3s-5r-nlp-mak-reinforce-sil-council/f38c5e649f3b4c14b7e761356bf9808a</t>
         </is>
       </c>
-      <c r="C3" s="7" t="n"/>
+      <c r="C3" s="8" t="n"/>
       <c r="D3" s="7" t="n"/>
       <c r="E3" s="7" t="n"/>
       <c r="F3" s="7" t="n"/>
-      <c r="G3" s="4" t="n">
+      <c r="G3" s="5" t="n">
         <v>0.0001</v>
       </c>
-      <c r="H3" s="5" t="n">
+      <c r="H3" s="6" t="n">
         <v>300</v>
       </c>
       <c r="I3" s="7" t="inlineStr">
@@ -735,16 +744,16 @@
           <t>(5, 3, 2, 1280)</t>
         </is>
       </c>
-      <c r="J3" s="5" t="n">
+      <c r="J3" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="K3" s="5" t="n">
+      <c r="K3" s="6" t="n">
         <v>1024</v>
       </c>
-      <c r="L3" s="5" t="n">
+      <c r="L3" s="6" t="n">
         <v>10240</v>
       </c>
-      <c r="M3" s="5" t="n">
+      <c r="M3" s="6" t="n">
         <v>128</v>
       </c>
       <c r="N3" s="7" t="inlineStr">
@@ -757,22 +766,22 @@
           <t>{'risk': 0.9, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
         </is>
       </c>
-      <c r="P3" s="5" t="n">
+      <c r="P3" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="Q3" s="5" t="n">
-        <v>100</v>
-      </c>
-      <c r="R3" s="5" t="n">
-        <v>100</v>
-      </c>
-      <c r="S3" s="5" t="n">
+      <c r="Q3" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="R3" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="S3" s="6" t="n">
         <v>1000</v>
       </c>
-      <c r="T3" s="5" t="n">
+      <c r="T3" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="U3" s="5" t="n">
+      <c r="U3" s="6" t="n">
         <v>9</v>
       </c>
       <c r="V3" s="7" t="inlineStr">
@@ -812,14 +821,14 @@
           <t>https://www.comet.com/redsnic/mak-3s-5r-nlp-mak-reinforce-sil-council/8acbba12fca44965a958068865eddd5e</t>
         </is>
       </c>
-      <c r="C4" s="7" t="n"/>
+      <c r="C4" s="8" t="n"/>
       <c r="D4" s="7" t="n"/>
       <c r="E4" s="7" t="n"/>
       <c r="F4" s="7" t="n"/>
-      <c r="G4" s="4" t="n">
+      <c r="G4" s="5" t="n">
         <v>0.0001</v>
       </c>
-      <c r="H4" s="5" t="n">
+      <c r="H4" s="6" t="n">
         <v>300</v>
       </c>
       <c r="I4" s="7" t="inlineStr">
@@ -827,16 +836,16 @@
           <t>(5, 3, 2, 1280)</t>
         </is>
       </c>
-      <c r="J4" s="5" t="n">
+      <c r="J4" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="K4" s="5" t="n">
+      <c r="K4" s="6" t="n">
         <v>1024</v>
       </c>
-      <c r="L4" s="5" t="n">
+      <c r="L4" s="6" t="n">
         <v>10240</v>
       </c>
-      <c r="M4" s="5" t="n">
+      <c r="M4" s="6" t="n">
         <v>128</v>
       </c>
       <c r="N4" s="7" t="inlineStr">
@@ -849,22 +858,22 @@
           <t>{'risk': 0.9, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
         </is>
       </c>
-      <c r="P4" s="5" t="n">
+      <c r="P4" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="Q4" s="5" t="n">
-        <v>100</v>
-      </c>
-      <c r="R4" s="5" t="n">
-        <v>100</v>
-      </c>
-      <c r="S4" s="5" t="n">
+      <c r="Q4" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="R4" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="S4" s="6" t="n">
         <v>1000</v>
       </c>
-      <c r="T4" s="5" t="n">
+      <c r="T4" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="U4" s="5" t="n">
+      <c r="U4" s="6" t="n">
         <v>9</v>
       </c>
       <c r="V4" s="7" t="inlineStr">
@@ -904,14 +913,14 @@
           <t>https://www.comet.com/redsnic/mak-3s-5r-nlp-mak-reinforce-sil-council/723c3786245a46d2a0e8bad5347f9870</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n"/>
+      <c r="C5" s="8" t="n"/>
       <c r="D5" s="7" t="n"/>
       <c r="E5" s="7" t="n"/>
       <c r="F5" s="7" t="n"/>
-      <c r="G5" s="4" t="n">
+      <c r="G5" s="5" t="n">
         <v>0.0001</v>
       </c>
-      <c r="H5" s="5" t="n">
+      <c r="H5" s="6" t="n">
         <v>300</v>
       </c>
       <c r="I5" s="7" t="inlineStr">
@@ -919,16 +928,16 @@
           <t>(5, 3, 2, 1280)</t>
         </is>
       </c>
-      <c r="J5" s="5" t="n">
+      <c r="J5" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="K5" s="5" t="n">
+      <c r="K5" s="6" t="n">
         <v>1024</v>
       </c>
-      <c r="L5" s="5" t="n">
+      <c r="L5" s="6" t="n">
         <v>10240</v>
       </c>
-      <c r="M5" s="5" t="n">
+      <c r="M5" s="6" t="n">
         <v>128</v>
       </c>
       <c r="N5" s="7" t="inlineStr">
@@ -941,22 +950,22 @@
           <t>{'risk': 0.9, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
         </is>
       </c>
-      <c r="P5" s="5" t="n">
+      <c r="P5" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="Q5" s="5" t="n">
-        <v>100</v>
-      </c>
-      <c r="R5" s="5" t="n">
-        <v>100</v>
-      </c>
-      <c r="S5" s="5" t="n">
+      <c r="Q5" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="R5" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="S5" s="6" t="n">
         <v>1000</v>
       </c>
-      <c r="T5" s="5" t="n">
+      <c r="T5" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="U5" s="5" t="n">
+      <c r="U5" s="6" t="n">
         <v>9</v>
       </c>
       <c r="V5" s="7" t="inlineStr">
@@ -996,14 +1005,14 @@
           <t>https://www.comet.com/redsnic/mak-3s-5r-nlp-mak-reinforce-sil-council/ea188c34e16046d99f41908c24e551d2</t>
         </is>
       </c>
-      <c r="C6" s="7" t="n"/>
+      <c r="C6" s="8" t="n"/>
       <c r="D6" s="7" t="n"/>
       <c r="E6" s="7" t="n"/>
       <c r="F6" s="7" t="n"/>
-      <c r="G6" s="4" t="n">
+      <c r="G6" s="5" t="n">
         <v>0.0001</v>
       </c>
-      <c r="H6" s="5" t="n">
+      <c r="H6" s="6" t="n">
         <v>300</v>
       </c>
       <c r="I6" s="7" t="inlineStr">
@@ -1011,16 +1020,16 @@
           <t>(5, 3, 2, 1280)</t>
         </is>
       </c>
-      <c r="J6" s="5" t="n">
+      <c r="J6" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="K6" s="5" t="n">
+      <c r="K6" s="6" t="n">
         <v>1024</v>
       </c>
-      <c r="L6" s="5" t="n">
+      <c r="L6" s="6" t="n">
         <v>10240</v>
       </c>
-      <c r="M6" s="5" t="n">
+      <c r="M6" s="6" t="n">
         <v>128</v>
       </c>
       <c r="N6" s="7" t="inlineStr">
@@ -1033,22 +1042,22 @@
           <t>{'risk': 0.9, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
         </is>
       </c>
-      <c r="P6" s="5" t="n">
+      <c r="P6" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="Q6" s="5" t="n">
-        <v>100</v>
-      </c>
-      <c r="R6" s="5" t="n">
-        <v>100</v>
-      </c>
-      <c r="S6" s="5" t="n">
+      <c r="Q6" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="R6" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="S6" s="6" t="n">
         <v>1000</v>
       </c>
-      <c r="T6" s="5" t="n">
+      <c r="T6" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="U6" s="5" t="n">
+      <c r="U6" s="6" t="n">
         <v>9</v>
       </c>
       <c r="V6" s="7" t="inlineStr">
@@ -1088,14 +1097,14 @@
           <t>https://www.comet.com/redsnic/mak-3s-5r-nlp-mak-reinforce-sil-council/6fc160a2095344de8435de464f252f92</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n"/>
+      <c r="C7" s="8" t="n"/>
       <c r="D7" s="7" t="n"/>
       <c r="E7" s="7" t="n"/>
       <c r="F7" s="7" t="n"/>
-      <c r="G7" s="4" t="n">
+      <c r="G7" s="5" t="n">
         <v>0.0001</v>
       </c>
-      <c r="H7" s="5" t="n">
+      <c r="H7" s="6" t="n">
         <v>300</v>
       </c>
       <c r="I7" s="7" t="inlineStr">
@@ -1103,16 +1112,16 @@
           <t>(5, 3, 2, 1280)</t>
         </is>
       </c>
-      <c r="J7" s="5" t="n">
+      <c r="J7" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="K7" s="5" t="n">
+      <c r="K7" s="6" t="n">
         <v>1024</v>
       </c>
-      <c r="L7" s="5" t="n">
+      <c r="L7" s="6" t="n">
         <v>10240</v>
       </c>
-      <c r="M7" s="5" t="n">
+      <c r="M7" s="6" t="n">
         <v>128</v>
       </c>
       <c r="N7" s="7" t="inlineStr">
@@ -1125,22 +1134,22 @@
           <t>{'risk': 0.9, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
         </is>
       </c>
-      <c r="P7" s="5" t="n">
+      <c r="P7" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="Q7" s="5" t="n">
-        <v>100</v>
-      </c>
-      <c r="R7" s="5" t="n">
-        <v>100</v>
-      </c>
-      <c r="S7" s="5" t="n">
+      <c r="Q7" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="R7" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="S7" s="6" t="n">
         <v>1000</v>
       </c>
-      <c r="T7" s="5" t="n">
+      <c r="T7" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="U7" s="5" t="n">
+      <c r="U7" s="6" t="n">
         <v>9</v>
       </c>
       <c r="V7" s="7" t="inlineStr">
@@ -1180,14 +1189,14 @@
           <t>https://www.comet.com/redsnic/mak-3s-5r-nlp-mak-reinforce-sil-council/f989d205eaca41469ebb7fed8d5b1cf7</t>
         </is>
       </c>
-      <c r="C8" s="7" t="n"/>
+      <c r="C8" s="8" t="n"/>
       <c r="D8" s="7" t="n"/>
       <c r="E8" s="7" t="n"/>
       <c r="F8" s="7" t="n"/>
-      <c r="G8" s="4" t="n">
+      <c r="G8" s="5" t="n">
         <v>0.0001</v>
       </c>
-      <c r="H8" s="5" t="n">
+      <c r="H8" s="6" t="n">
         <v>300</v>
       </c>
       <c r="I8" s="7" t="inlineStr">
@@ -1195,16 +1204,16 @@
           <t>(5, 3, 2, 1280)</t>
         </is>
       </c>
-      <c r="J8" s="5" t="n">
+      <c r="J8" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="K8" s="5" t="n">
+      <c r="K8" s="6" t="n">
         <v>1024</v>
       </c>
-      <c r="L8" s="5" t="n">
+      <c r="L8" s="6" t="n">
         <v>10240</v>
       </c>
-      <c r="M8" s="5" t="n">
+      <c r="M8" s="6" t="n">
         <v>128</v>
       </c>
       <c r="N8" s="7" t="inlineStr">
@@ -1217,22 +1226,22 @@
           <t>{'risk': 0.9, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
         </is>
       </c>
-      <c r="P8" s="5" t="n">
+      <c r="P8" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="Q8" s="5" t="n">
-        <v>100</v>
-      </c>
-      <c r="R8" s="5" t="n">
-        <v>100</v>
-      </c>
-      <c r="S8" s="5" t="n">
+      <c r="Q8" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="R8" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="S8" s="6" t="n">
         <v>1000</v>
       </c>
-      <c r="T8" s="5" t="n">
+      <c r="T8" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="U8" s="5" t="n">
+      <c r="U8" s="6" t="n">
         <v>9</v>
       </c>
       <c r="V8" s="7" t="inlineStr">
@@ -1272,14 +1281,14 @@
           <t>https://www.comet.com/redsnic/mak-3s-5r-nlp-mak-reinforce-sil-council/81d3d74688564160a7264f91accc5987</t>
         </is>
       </c>
-      <c r="C9" s="7" t="n"/>
+      <c r="C9" s="8" t="n"/>
       <c r="D9" s="7" t="n"/>
       <c r="E9" s="7" t="n"/>
       <c r="F9" s="7" t="n"/>
-      <c r="G9" s="4" t="n">
+      <c r="G9" s="5" t="n">
         <v>0.0001</v>
       </c>
-      <c r="H9" s="5" t="n">
+      <c r="H9" s="6" t="n">
         <v>300</v>
       </c>
       <c r="I9" s="7" t="inlineStr">
@@ -1287,16 +1296,16 @@
           <t>(5, 3, 2, 1280)</t>
         </is>
       </c>
-      <c r="J9" s="5" t="n">
+      <c r="J9" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="K9" s="5" t="n">
+      <c r="K9" s="6" t="n">
         <v>1024</v>
       </c>
-      <c r="L9" s="5" t="n">
+      <c r="L9" s="6" t="n">
         <v>10240</v>
       </c>
-      <c r="M9" s="5" t="n">
+      <c r="M9" s="6" t="n">
         <v>128</v>
       </c>
       <c r="N9" s="7" t="inlineStr">
@@ -1309,22 +1318,22 @@
           <t>{'risk': 0.9, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
         </is>
       </c>
-      <c r="P9" s="5" t="n">
+      <c r="P9" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="Q9" s="5" t="n">
-        <v>100</v>
-      </c>
-      <c r="R9" s="5" t="n">
-        <v>100</v>
-      </c>
-      <c r="S9" s="5" t="n">
+      <c r="Q9" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="R9" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="S9" s="6" t="n">
         <v>1000</v>
       </c>
-      <c r="T9" s="5" t="n">
+      <c r="T9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="U9" s="5" t="n">
+      <c r="U9" s="6" t="n">
         <v>9</v>
       </c>
       <c r="V9" s="7" t="inlineStr">
@@ -1364,14 +1373,14 @@
           <t>https://www.comet.com/redsnic/mak-3s-5r-nlp-mak-reinforce-sil-council/6f5b66c831d041319350482675b0ea63</t>
         </is>
       </c>
-      <c r="C10" s="7" t="n"/>
+      <c r="C10" s="8" t="n"/>
       <c r="D10" s="7" t="n"/>
       <c r="E10" s="7" t="n"/>
       <c r="F10" s="7" t="n"/>
-      <c r="G10" s="4" t="n">
+      <c r="G10" s="5" t="n">
         <v>0.0001</v>
       </c>
-      <c r="H10" s="5" t="n">
+      <c r="H10" s="6" t="n">
         <v>300</v>
       </c>
       <c r="I10" s="7" t="inlineStr">
@@ -1379,16 +1388,16 @@
           <t>(5, 3, 2, 1280)</t>
         </is>
       </c>
-      <c r="J10" s="5" t="n">
+      <c r="J10" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="K10" s="5" t="n">
+      <c r="K10" s="6" t="n">
         <v>1024</v>
       </c>
-      <c r="L10" s="5" t="n">
+      <c r="L10" s="6" t="n">
         <v>10240</v>
       </c>
-      <c r="M10" s="5" t="n">
+      <c r="M10" s="6" t="n">
         <v>128</v>
       </c>
       <c r="N10" s="7" t="inlineStr">
@@ -1401,22 +1410,22 @@
           <t>{'risk': 0.9, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
         </is>
       </c>
-      <c r="P10" s="5" t="n">
+      <c r="P10" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="Q10" s="5" t="n">
-        <v>100</v>
-      </c>
-      <c r="R10" s="5" t="n">
-        <v>100</v>
-      </c>
-      <c r="S10" s="5" t="n">
+      <c r="Q10" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="R10" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="S10" s="6" t="n">
         <v>1000</v>
       </c>
-      <c r="T10" s="5" t="n">
+      <c r="T10" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="U10" s="5" t="n">
+      <c r="U10" s="6" t="n">
         <v>9</v>
       </c>
       <c r="V10" s="7" t="inlineStr">
@@ -1456,7 +1465,7 @@
           <t>https://www.comet.com/redsnic/mak-3s-5r-nlp-mak-reinforce-sil-council/c852fd1b664f46fd91e1491bf98d1f16</t>
         </is>
       </c>
-      <c r="C11" s="6" t="n">
+      <c r="C11" s="4" t="n">
         <v>300</v>
       </c>
       <c r="D11" s="7" t="inlineStr">
@@ -1474,10 +1483,10 @@
           <t>Extremely good loss. NLPs dominated!</t>
         </is>
       </c>
-      <c r="G11" s="4" t="n">
+      <c r="G11" s="5" t="n">
         <v>0.0001</v>
       </c>
-      <c r="H11" s="5" t="n">
+      <c r="H11" s="6" t="n">
         <v>300</v>
       </c>
       <c r="I11" s="7" t="inlineStr">
@@ -1485,16 +1494,16 @@
           <t>(5, 3, 2, 1280)</t>
         </is>
       </c>
-      <c r="J11" s="5" t="n">
+      <c r="J11" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="K11" s="5" t="n">
+      <c r="K11" s="6" t="n">
         <v>1024</v>
       </c>
-      <c r="L11" s="5" t="n">
+      <c r="L11" s="6" t="n">
         <v>10240</v>
       </c>
-      <c r="M11" s="5" t="n">
+      <c r="M11" s="6" t="n">
         <v>128</v>
       </c>
       <c r="N11" s="7" t="inlineStr">
@@ -1507,22 +1516,22 @@
           <t>{'risk': 0.9, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
         </is>
       </c>
-      <c r="P11" s="5" t="n">
+      <c r="P11" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="Q11" s="5" t="n">
-        <v>100</v>
-      </c>
-      <c r="R11" s="5" t="n">
-        <v>100</v>
-      </c>
-      <c r="S11" s="5" t="n">
+      <c r="Q11" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="R11" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="S11" s="6" t="n">
         <v>1000</v>
       </c>
-      <c r="T11" s="5" t="n">
+      <c r="T11" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="U11" s="5" t="n">
+      <c r="U11" s="6" t="n">
         <v>9</v>
       </c>
       <c r="V11" s="7" t="inlineStr">
@@ -1551,96 +1560,202 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+    <row r="12" ht="19.5" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>2025-12-18 17:21:19</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>https://www.comet.com/redsnic/mak-3s-5r-nlp-mak-reinforce-sil-council/f551ee014f1e499c8298d050de4afb18</t>
         </is>
       </c>
-      <c r="G12" t="n">
+      <c r="C12" s="4" t="n">
+        <v>300</v>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>Extremely good loss. NLPs dominated!</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="n">
         <v>0.0001</v>
       </c>
-      <c r="H12" t="n">
+      <c r="H12" s="4" t="n">
         <v>300</v>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="I12" s="7" t="inlineStr">
         <is>
           <t>(5, 3, 2, 1280)</t>
         </is>
       </c>
-      <c r="J12" t="n">
+      <c r="J12" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="K12" t="n">
+      <c r="K12" s="4" t="n">
         <v>1024</v>
       </c>
-      <c r="L12" t="n">
+      <c r="L12" s="4" t="n">
         <v>10240</v>
       </c>
-      <c r="M12" t="n">
+      <c r="M12" s="4" t="n">
         <v>128</v>
       </c>
-      <c r="N12" t="inlineStr">
+      <c r="N12" s="7" t="inlineStr">
         <is>
           <t>{'entropy_weight': 0.001, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr">
+      <c r="O12" s="7" t="inlineStr">
         <is>
           <t>{'risk': 0.9, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
         </is>
       </c>
-      <c r="P12" t="n">
+      <c r="P12" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="Q12" t="n">
-        <v>100</v>
-      </c>
-      <c r="R12" t="n">
-        <v>100</v>
-      </c>
-      <c r="S12" t="n">
+      <c r="Q12" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="R12" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="S12" s="4" t="n">
         <v>1000</v>
       </c>
-      <c r="T12" t="n">
+      <c r="T12" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="U12" t="n">
+      <c r="U12" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="V12" t="inlineStr">
+      <c r="V12" s="7" t="inlineStr">
         <is>
           <t>{'type': 'lognormal_1D'}</t>
         </is>
       </c>
-      <c r="W12" t="inlineStr">
+      <c r="W12" s="7" t="inlineStr">
         <is>
           <t>{'structure': 2.0, 'continuous': 1.0, 'discrete': 0.0, 'input_influence': 0.0}</t>
         </is>
       </c>
-      <c r="X12" t="inlineStr">
+      <c r="X12" s="7" t="inlineStr">
         <is>
           <t>{'target_entropy_ratio_to_max': np.float64(0.35679185088982296), 'initial_temperature': 1.0, 'rate': 0.0, 'current_temperature': 1.0}</t>
         </is>
       </c>
-      <c r="Y12" t="inlineStr">
+      <c r="Y12" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="Z12" t="inlineStr">
+      <c r="Z12" s="7" t="inlineStr">
+        <is>
+          <t>{'sil_loss_weight': 1.0, 'sil_use_adaptive_baseline': False, 'sil_baseline_annealing_rate': 0.95}</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2025-12-19 10:07:58</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/redsnic/mak-3s-5r-nlp-mak-reinforce-sil-council/7093031822e14ee898ecbd482851264f</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="H13" t="n">
+        <v>300</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>(5, 3, 2, 1280)</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>5</v>
+      </c>
+      <c r="K13" t="n">
+        <v>1024</v>
+      </c>
+      <c r="L13" t="n">
+        <v>10240</v>
+      </c>
+      <c r="M13" t="n">
+        <v>128</v>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>{'entropy_weight': 0.001, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>{'risk': 0.9, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
+        </is>
+      </c>
+      <c r="P13" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>100</v>
+      </c>
+      <c r="R13" t="n">
+        <v>100</v>
+      </c>
+      <c r="S13" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T13" t="n">
+        <v>1</v>
+      </c>
+      <c r="U13" t="n">
+        <v>9</v>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>{'type': 'lognormal_1D'}</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>{'structure': 2.0, 'continuous': 1.0, 'discrete': 0.0, 'input_influence': 0.0}</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>{'target_entropy_ratio_to_max': np.float64(0.35679185088982296), 'initial_temperature': 1.0, 'rate': 0.0, 'current_temperature': 1.0}</t>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Z13" t="inlineStr">
         <is>
           <t>{'sil_loss_weight': 1.0, 'sil_use_adaptive_baseline': False, 'sil_baseline_annealing_rate': 0.95}</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Z12"/>
+  <autoFilter ref="A1:Z13"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>